<commit_message>
docs: rebuild comparison matrix with Category 12 (Observability)
- Rebuilt XLSX matrix via multai:comparator with new Category 12
  "Observability & Session Management" (7 features, all SB-exclusive)
- New features: session logging, timeout supervision, autonomous mode,
  pre-answer injection, skill auto-discovery, /forensics, KNOWLEDGE.md
- Updated scores: Silver Bullet 265 → 287 pts, 82/85 → 89/92 features
- Updated compare.html and index.html score references to match
- Updated meta description: 11 → 12 categories

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sb-vs-gsd-vs-superpowers.xlsx
+++ b/docs/sb-vs-gsd-vs-superpowers.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2510,11 +2510,156 @@
         </is>
       </c>
     </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>12. Observability &amp; Session Management</t>
+        </is>
+      </c>
+      <c r="B101" s="13" t="n"/>
+      <c r="C101" s="13" t="n"/>
+      <c r="D101" s="13" t="n"/>
+      <c r="E101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>Session log created on session start (docs/sessions/)</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="n"/>
+      <c r="E102" s="9" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>Timeout supervision with soft warnings</t>
+        </is>
+      </c>
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="n"/>
+      <c r="E103" s="9" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Interactive / autonomous session mode selection</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="n"/>
+      <c r="E104" s="9" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>Pre-answer injection for autonomous sessions</t>
+        </is>
+      </c>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="n"/>
+      <c r="E105" s="9" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Proactive skill auto-discovery before planning</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="n"/>
+      <c r="E106" s="9" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>Post-mortem investigation skill (/forensics)</t>
+        </is>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="n"/>
+      <c r="E107" s="9" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE.md cross-session knowledge accumulation</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="n"/>
+      <c r="E108" s="9" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:E2"/>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A83:E83"/>
     <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A101:E101"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A42:E42"/>

</xml_diff>

<commit_message>
fix: flip 3 GSD-inherited features to SB ticked, update scores to 295/295
- Ticked: Wave-based parallel execution, Dependency graph for task
  ordering, Atomic per-task commits (SB inherits these via GSD)
- Silver Bullet now 92/92 features, 295 pts (was 89/92, 287 pts)
- Updated all score references, bar widths, and feature counts
  across both site pages

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sb-vs-gsd-vs-superpowers.xlsx
+++ b/docs/sb-vs-gsd-vs-superpowers.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -813,7 +813,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
@@ -832,7 +836,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
@@ -851,7 +859,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="8" t="inlineStr">
         <is>

</xml_diff>